<commit_message>
Block 2 Fallback Integration and Execution
</commit_message>
<xml_diff>
--- a/results/block1_results/Diseased_14/dataset_RCA_Diseased_14.xlsx
+++ b/results/block1_results/Diseased_14/dataset_RCA_Diseased_14.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H758"/>
+  <dimension ref="A1:H760"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23053,7 +23053,7 @@
       </c>
       <c r="G754" t="inlineStr">
         <is>
-          <t>Endpoint</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="H754" t="n">
@@ -23070,24 +23070,24 @@
         </is>
       </c>
       <c r="C755" t="n">
-        <v>189.3590240478516</v>
+        <v>202.0729370117188</v>
       </c>
       <c r="D755" t="n">
-        <v>223.6087036132812</v>
+        <v>219.0033569335938</v>
       </c>
       <c r="E755" t="n">
-        <v>-148.8290863037109</v>
+        <v>-152.3894500732422</v>
       </c>
       <c r="F755" t="n">
-        <v>0.5072876503416086</v>
+        <v>0.5698341079691279</v>
       </c>
       <c r="G755" t="inlineStr">
         <is>
-          <t>Endpoint</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="H755" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="756">
@@ -23100,24 +23100,24 @@
         </is>
       </c>
       <c r="C756" t="n">
-        <v>189.3731842041016</v>
+        <v>202.1583251953125</v>
       </c>
       <c r="D756" t="n">
-        <v>223.5946350097656</v>
+        <v>219.0409698486328</v>
       </c>
       <c r="E756" t="n">
-        <v>-148.8196411132812</v>
+        <v>-152.3893127441406</v>
       </c>
       <c r="F756" t="n">
-        <v>0.5165311662965</v>
+        <v>0.6163618775446726</v>
       </c>
       <c r="G756" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Endpoint</t>
         </is>
       </c>
       <c r="H756" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="757">
@@ -23130,20 +23130,20 @@
         </is>
       </c>
       <c r="C757" t="n">
-        <v>189.3702239990234</v>
+        <v>189.3590240478516</v>
       </c>
       <c r="D757" t="n">
-        <v>223.5768890380859</v>
+        <v>223.6087036132812</v>
       </c>
       <c r="E757" t="n">
-        <v>-148.8218078613281</v>
+        <v>-148.8290863037109</v>
       </c>
       <c r="F757" t="n">
-        <v>0.522315923721927</v>
+        <v>0.5072876503416086</v>
       </c>
       <c r="G757" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Endpoint</t>
         </is>
       </c>
       <c r="H757" t="n">
@@ -23160,23 +23160,83 @@
         </is>
       </c>
       <c r="C758" t="n">
-        <v>189.2925720214844</v>
+        <v>189.3731842041016</v>
       </c>
       <c r="D758" t="n">
-        <v>223.4728851318359</v>
+        <v>223.5946350097656</v>
       </c>
       <c r="E758" t="n">
-        <v>-148.8752899169922</v>
+        <v>-148.8196411132812</v>
       </c>
       <c r="F758" t="n">
-        <v>0.5570543662403887</v>
+        <v>0.5165311662965</v>
       </c>
       <c r="G758" t="inlineStr">
         <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="H758" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="n">
+        <v>14</v>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>RCA</t>
+        </is>
+      </c>
+      <c r="C759" t="n">
+        <v>189.3875885009766</v>
+      </c>
+      <c r="D759" t="n">
+        <v>223.5947113037109</v>
+      </c>
+      <c r="E759" t="n">
+        <v>-148.8191833496094</v>
+      </c>
+      <c r="F759" t="n">
+        <v>0.5130665633445103</v>
+      </c>
+      <c r="G759" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="H759" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="n">
+        <v>14</v>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>RCA</t>
+        </is>
+      </c>
+      <c r="C760" t="n">
+        <v>189.4791717529297</v>
+      </c>
+      <c r="D760" t="n">
+        <v>223.61865234375</v>
+      </c>
+      <c r="E760" t="n">
+        <v>-148.7881164550781</v>
+      </c>
+      <c r="F760" t="n">
+        <v>0.4690713717457025</v>
+      </c>
+      <c r="G760" t="inlineStr">
+        <is>
           <t>Endpoint</t>
         </is>
       </c>
-      <c r="H758" t="n">
+      <c r="H760" t="n">
         <v>19</v>
       </c>
     </row>

</xml_diff>